<commit_message>
results: re-evaluate with extended PA metric set (jaccard_pa + 10 more)
Re-ran scripts/evaluate.py on existing pickled predictions to populate
jaccard_pa, example/macro/micro {precision,recall,f1}_pa, afrd_pa, and
mfrd_pa in PA evaluation CSVs. Original CSVs only had the 7 legacy PA
metrics (abs/aabs/rec/arec/f1_pa/subset0_1_pa/hamming_accuracy_pa).

Covers 5 source dirs feeding paper_revision/build_panels.py FOLDER_MAP:
  - results/20260514_v2 (RF, 9 original-paper datasets)
  - results/full_birds (RF) and results/full_birds_lgbm
  - results/full_medical_split (RF) and results/full_medical_lgbm_split

Regenerated per-dataset summary tables in:
  final_20260514_v2_summary, full_birds_summary, full_birds_lgbm_summary,
  full_medical_summary, full_medical_lgbm_summary

Not covered: results/full_enron_split_summary — the RF enron pickles are
no longer on disk (only evaluation CSVs remain), so jaccard_pa for enron
RF cannot be recovered without retraining.
</commit_message>
<xml_diff>
--- a/results/20260514_v2/evaluation_VirusPseAAC_noisy_0.0_ecc.xlsx
+++ b/results/20260514_v2/evaluation_VirusPseAAC_noisy_0.0_ecc.xlsx
@@ -981,12 +981,8 @@
           <t>auc_macro</t>
         </is>
       </c>
-      <c r="H20" t="n">
-        <v>0.79055</v>
-      </c>
-      <c r="I20" t="n">
-        <v>0.05088</v>
-      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">

</xml_diff>